<commit_message>
Gestores: aplica mudanças do arquivo dos professores e adiciona TCLE
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01AahsCeqM2DTecRKsTTfJbG
</commit_message>
<xml_diff>
--- a/kobo/gestores_semana3_diagnostico.xlsx
+++ b/kobo/gestores_semana3_diagnostico.xlsx
@@ -424,7 +424,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J89"/>
+  <dimension ref="A1:J96"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -579,12 +579,12 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>identificacao</t>
+          <t>tcle</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Identificação (igual à Semana 1)</t>
+          <t>Termo de Consentimento</t>
         </is>
       </c>
       <c r="D6" t="inlineStr"/>
@@ -598,25 +598,21 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>id_escola</t>
+          <t>tcle_texto</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Nome do local de atuação</t>
+          <t>TERMO DE CONSENTIMENTO LIVRE E ESCLARECIDO. Você está sendo convidado(a) a responder este Diagnóstico Socioambiental, Climático e de Educação Ambiental. A participação é voluntária: você pode recusar ou interromper a qualquer momento, sem qualquer prejuízo. As informações fornecidas, inclusive seus dados pessoais e de identificação (nome, função, local de atuação), serão tratadas com sigilo, NÃO serão compartilhadas com terceiros de forma que identifique você ou o seu local de atuação e serão utilizadas apenas para compor um banco de dados do projeto. Eventuais resultados e relatórios serão apresentados somente de forma agregada, sem identificar pessoas. O tratamento dos dados segue a Lei Geral de Proteção de Dados (Lei nº 13.709/2018). Em caso de dúvidas, procure a equipe responsável pelo projeto.</t>
         </is>
       </c>
       <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+      <c r="E7" t="inlineStr"/>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr"/>
@@ -626,58 +622,54 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one concordo</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>id_inep</t>
+          <t>tcle_consentimento</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Código INEP (apenas se for local; 8 dígitos)</t>
+          <t>Li o termo acima e concordo em participar e em ter minhas respostas e meus dados utilizados no banco de dados do projeto, nos termos descritos.</t>
         </is>
       </c>
       <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr">
-        <is>
-          <t>regex(., '^[0-9]{8}$')</t>
-        </is>
-      </c>
-      <c r="I8" t="inlineStr">
-        <is>
-          <t>O código INEP deve ter 8 dígitos.</t>
-        </is>
-      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr"/>
       <c r="J8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>id_nome</t>
+          <t>tcle_recusa</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Seu nome</t>
+          <t>Sem o seu consentimento não é possível continuar. Obrigado(a) pelo seu tempo! Você pode encerrar o formulário.</t>
         </is>
       </c>
       <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F9" t="inlineStr"/>
+      <c r="E9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>${tcle_consentimento} = 'nao_concordo'</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr"/>
       <c r="I9" t="inlineStr"/>
@@ -707,17 +699,21 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>etapa4</t>
+          <t>conteudo</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Etapa 4 — Riscos Climáticos</t>
+          <t>Diagnóstico</t>
         </is>
       </c>
       <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr"/>
-      <c r="F11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>${tcle_consentimento} = 'concordo'</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr"/>
       <c r="I11" t="inlineStr"/>
@@ -726,25 +722,21 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>select_multiple ameacas</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>q4_1</t>
+          <t>identificacao</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Q4.1. Quais ameaças/eventos climáticos já afetaram (ou podem afetar) o local/comunidade?</t>
+          <t>Identificação (igual à Semana 1)</t>
         </is>
       </c>
       <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+      <c r="E12" t="inlineStr"/>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr"/>
@@ -759,21 +751,21 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>q4_1_outro</t>
+          <t>id_escola</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Nome do local de atuação</t>
         </is>
       </c>
       <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
-      <c r="F13" t="inlineStr">
-        <is>
-          <t>selected(${q4_1}, 'outro')</t>
-        </is>
-      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr"/>
       <c r="I13" t="inlineStr"/>
@@ -782,25 +774,33 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>q4_2</t>
+          <t>id_inep</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Q4.2. A comunidade percebe mudanças no padrão climático local ao longo dos anos?</t>
+          <t>Código INEP (apenas se for local; 8 dígitos)</t>
         </is>
       </c>
       <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr"/>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
-      <c r="I14" t="inlineStr"/>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>regex(., '^[0-9]{8}$')</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>O código INEP deve ter 8 dígitos.</t>
+        </is>
+      </c>
       <c r="J14" t="inlineStr"/>
     </row>
     <row r="15">
@@ -811,30 +811,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>q4_3</t>
+          <t>id_nome</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Q4.3. Que mudanças são percebidas?</t>
-        </is>
-      </c>
-      <c r="D15" t="inlineStr">
-        <is>
-          <t>Registre como percepção da comunidade — o relatório final não converterá isso em dado técnico comprovado.</t>
-        </is>
-      </c>
-      <c r="E15" t="inlineStr"/>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>${q4_2}='sim'</t>
-        </is>
-      </c>
-      <c r="G15" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+          <t>Seu nome</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr"/>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr"/>
+      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr"/>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
@@ -842,26 +834,14 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>select_multiple base_percepcao</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>q4_4</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>Q4.4. Com base em quê essa percepção se formou?</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
       <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr"/>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>${q4_2}='sim'</t>
-        </is>
-      </c>
+      <c r="F16" t="inlineStr"/>
       <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr"/>
       <c r="I16" t="inlineStr"/>
@@ -870,17 +850,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>select_multiple fontes_risco</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>q4_5</t>
+          <t>etapa4</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Q4.5. Existem fontes técnicas de informação sobre riscos consultadas pelo local?</t>
+          <t>Etapa 4 — Riscos Climáticos</t>
         </is>
       </c>
       <c r="D17" t="inlineStr"/>
@@ -894,26 +874,26 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple ameacas</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>q4_5_outro</t>
+          <t>q4_1</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q4.1. Quais ameaças/eventos climáticos já afetaram (ou podem afetar) o local/comunidade?</t>
         </is>
       </c>
       <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
-      <c r="F18" t="inlineStr">
-        <is>
-          <t>selected(${q4_5}, 'outro')</t>
-        </is>
-      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr"/>
       <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr"/>
       <c r="I18" t="inlineStr"/>
@@ -922,22 +902,26 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>q4_6</t>
+          <t>q4_1_outro</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Q4.6. Seria necessário apoio técnico para avaliar melhor esses riscos?</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr"/>
-      <c r="F19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>selected(${q4_1}, 'outro')</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr"/>
       <c r="I19" t="inlineStr"/>
@@ -946,31 +930,23 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>q4_7</t>
+          <t>q4_2</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Q4.7. Apoio técnico para quê, especificamente?</t>
+          <t>Q4.2. A comunidade percebe mudanças no padrão climático local ao longo dos anos?</t>
         </is>
       </c>
       <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr"/>
-      <c r="F20" t="inlineStr">
-        <is>
-          <t>${q4_6}='sim'</t>
-        </is>
-      </c>
-      <c r="G20" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F20" t="inlineStr"/>
+      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr"/>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
@@ -983,17 +959,25 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>q4_8</t>
+          <t>q4_3</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Q4.8. Algum ator já mapeado poderia oferecer esse apoio? (informe o nome do ator, conforme Etapa 3)</t>
-        </is>
-      </c>
-      <c r="D21" t="inlineStr"/>
+          <t>Q4.3. Que mudanças são percebidas?</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>Registre como percepção da comunidade — o relatório final não converterá isso em dado técnico comprovado.</t>
+        </is>
+      </c>
       <c r="E21" t="inlineStr"/>
-      <c r="F21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>${q4_2}='sim'</t>
+        </is>
+      </c>
       <c r="G21" t="inlineStr">
         <is>
           <t>multiline</t>
@@ -1006,22 +990,26 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>select_multiple base_percepcao</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>risco</t>
+          <t>q4_4</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ficha de risco (RISK_*) — uma ficha para cada ameaça selecionada na Q4.1</t>
+          <t>Q4.4. Com base em quê essa percepção se formou?</t>
         </is>
       </c>
       <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr"/>
-      <c r="F22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>${q4_2}='sim'</t>
+        </is>
+      </c>
       <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr"/>
       <c r="I22" t="inlineStr"/>
@@ -1030,17 +1018,17 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_multiple fontes_risco</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>risco_nota</t>
+          <t>q4_5</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Preencha uma ficha por ameaça selecionada na Q4.1 (use "Adicionar" para cada nova). No sistema original as fichas são sugeridas automaticamente; aqui, escolha a ameaça abaixo.</t>
+          <t>Q4.5. Existem fontes técnicas de informação sobre riscos consultadas pelo local?</t>
         </is>
       </c>
       <c r="D23" t="inlineStr"/>
@@ -1054,26 +1042,26 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>select_one ameacas</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>risco_ameaca</t>
+          <t>q4_5_outro</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Ameaça/evento climático desta ficha</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
-      <c r="F24" t="inlineStr"/>
+      <c r="E24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>selected(${q4_5}, 'outro')</t>
+        </is>
+      </c>
       <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr"/>
       <c r="I24" t="inlineStr"/>
@@ -1082,26 +1070,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>risco_ameaca_outro</t>
+          <t>q4_6</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Q4.6. Seria necessário apoio técnico para avaliar melhor esses riscos?</t>
         </is>
       </c>
       <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr"/>
-      <c r="F25" t="inlineStr">
-        <is>
-          <t>${risco_ameaca}='outro'</t>
-        </is>
-      </c>
+      <c r="F25" t="inlineStr"/>
       <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr"/>
       <c r="I25" t="inlineStr"/>
@@ -1110,23 +1094,31 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>select_one sim_nao_nsabe</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>risco_ocorreu</t>
+          <t>q4_7</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Já ocorreu antes?</t>
+          <t>Q4.7. Apoio técnico para quê, especificamente?</t>
         </is>
       </c>
       <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr"/>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>${q4_6}='sim'</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H26" t="inlineStr"/>
       <c r="I26" t="inlineStr"/>
       <c r="J26" t="inlineStr"/>
@@ -1134,23 +1126,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>select_one afetou</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>risco_afetou</t>
+          <t>q4_8</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Afetou o local, a comunidade, ou ambos?</t>
+          <t>Q4.8. Algum ator já mapeado poderia oferecer esse apoio? (informe o nome do ator, conforme Etapa 3)</t>
         </is>
       </c>
       <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr"/>
       <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H27" t="inlineStr"/>
       <c r="I27" t="inlineStr"/>
       <c r="J27" t="inlineStr"/>
@@ -1158,17 +1154,17 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>select_one freq_risco</t>
+          <t>begin_repeat</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>risco_freq</t>
+          <t>risco</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Frequência</t>
+          <t>Ficha de risco (RISK_*) — uma ficha para cada ameaça selecionada na Q4.1</t>
         </is>
       </c>
       <c r="D28" t="inlineStr"/>
@@ -1182,53 +1178,49 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>risco_ano</t>
+          <t>risco_nota</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Ano da última ocorrência</t>
+          <t>Preencha uma ficha por ameaça selecionada na Q4.1 (use "Adicionar" para cada nova). No sistema original as fichas são sugeridas automaticamente; aqui, escolha a ameaça abaixo.</t>
         </is>
       </c>
       <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr"/>
       <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr"/>
-      <c r="H29" t="inlineStr">
-        <is>
-          <t>. = '' or regex(., '^[0-9]{4}$')</t>
-        </is>
-      </c>
-      <c r="I29" t="inlineStr">
-        <is>
-          <t>Informe um ano com 4 dígitos.</t>
-        </is>
-      </c>
+      <c r="H29" t="inlineStr"/>
+      <c r="I29" t="inlineStr"/>
       <c r="J29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one ameacas</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>risco_periodo</t>
+          <t>risco_ameaca</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Período do ano em que costuma ocorrer</t>
+          <t>Ameaça/evento climático desta ficha</t>
         </is>
       </c>
       <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr"/>
@@ -1238,22 +1230,26 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>select_multiple impacto_risco</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>risco_impactos</t>
+          <t>risco_ameaca_outro</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Impactos observados</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr"/>
-      <c r="F31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>${risco_ameaca}='outro'</t>
+        </is>
+      </c>
       <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr"/>
       <c r="I31" t="inlineStr"/>
@@ -1262,26 +1258,22 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one sim_nao_nsabe</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>risco_impactos_outro</t>
+          <t>risco_ocorreu</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Já ocorreu antes?</t>
         </is>
       </c>
       <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr"/>
-      <c r="F32" t="inlineStr">
-        <is>
-          <t>selected(${risco_impactos}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr"/>
       <c r="I32" t="inlineStr"/>
@@ -1290,27 +1282,23 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_one afetou</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>risco_impactos_desc</t>
+          <t>risco_afetou</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Descreva os impactos</t>
+          <t>Afetou o local, a comunidade, ou ambos?</t>
         </is>
       </c>
       <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr"/>
       <c r="F33" t="inlineStr"/>
-      <c r="G33" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr"/>
       <c r="I33" t="inlineStr"/>
       <c r="J33" t="inlineStr"/>
@@ -1318,17 +1306,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>select_multiple ativos</t>
+          <t>select_one freq_risco</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>risco_ativos</t>
+          <t>risco_freq</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ativos/estruturas expostos</t>
+          <t>Frequência</t>
         </is>
       </c>
       <c r="D34" t="inlineStr"/>
@@ -1347,40 +1335,44 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>risco_ativos_outro</t>
+          <t>risco_ano</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Ano da última ocorrência</t>
         </is>
       </c>
       <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr"/>
-      <c r="F35" t="inlineStr">
-        <is>
-          <t>selected(${risco_ativos}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr"/>
-      <c r="H35" t="inlineStr"/>
-      <c r="I35" t="inlineStr"/>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>. = '' or regex(., '^[0-9]{4}$')</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Informe um ano com 4 dígitos.</t>
+        </is>
+      </c>
       <c r="J35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>select_multiple grupos_exp</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>risco_grupos</t>
+          <t>risco_periodo</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Grupos expostos</t>
+          <t>Período do ano em que costuma ocorrer</t>
         </is>
       </c>
       <c r="D36" t="inlineStr"/>
@@ -1394,26 +1386,22 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple impacto_risco</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>risco_grupos_outro</t>
+          <t>risco_impactos</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Impactos observados</t>
         </is>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>selected(${risco_grupos}, 'outro')</t>
-        </is>
-      </c>
+      <c r="F37" t="inlineStr"/>
       <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr"/>
       <c r="I37" t="inlineStr"/>
@@ -1422,22 +1410,26 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>select_multiple cond_amplia</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>risco_condicoes</t>
+          <t>risco_impactos_outro</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Condições que podem ampliar dificuldades de proteção (não são características das pessoas — são condições do ambiente/organização)</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
-      <c r="F38" t="inlineStr"/>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>selected(${risco_impactos}, 'outro')</t>
+        </is>
+      </c>
       <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr"/>
       <c r="I38" t="inlineStr"/>
@@ -1451,22 +1443,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>risco_condicoes_outro</t>
+          <t>risco_impactos_desc</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Descreva os impactos</t>
         </is>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
-      <c r="F39" t="inlineStr">
-        <is>
-          <t>selected(${risco_condicoes}, 'outro')</t>
-        </is>
-      </c>
-      <c r="G39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr"/>
       <c r="J39" t="inlineStr"/>
@@ -1474,17 +1466,17 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>select_multiple cap_resp</t>
+          <t>select_multiple ativos</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>risco_capacidades</t>
+          <t>risco_ativos</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Capacidades de resposta já existentes</t>
+          <t>Ativos/estruturas expostos</t>
         </is>
       </c>
       <c r="D40" t="inlineStr"/>
@@ -1503,7 +1495,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>risco_capacidades_outro</t>
+          <t>risco_ativos_outro</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1515,7 +1507,7 @@
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="inlineStr">
         <is>
-          <t>selected(${risco_capacidades}, 'outro')</t>
+          <t>selected(${risco_ativos}, 'outro')</t>
         </is>
       </c>
       <c r="G41" t="inlineStr"/>
@@ -1526,17 +1518,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>select_one aval_cap</t>
+          <t>select_multiple grupos_exp</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>risco_aval_cap</t>
+          <t>risco_grupos</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Avaliação geral da capacidade de resposta</t>
+          <t>Grupos expostos</t>
         </is>
       </c>
       <c r="D42" t="inlineStr"/>
@@ -1550,22 +1542,26 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>select_one bma_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>risco_prob</t>
+          <t>risco_grupos_outro</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Probabilidade percebida (não é medição técnica)</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
-      <c r="F43" t="inlineStr"/>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>selected(${risco_grupos}, 'outro')</t>
+        </is>
+      </c>
       <c r="G43" t="inlineStr"/>
       <c r="H43" t="inlineStr"/>
       <c r="I43" t="inlineStr"/>
@@ -1574,17 +1570,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>select_one bma_ns</t>
+          <t>select_multiple cond_amplia</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>risco_grav</t>
+          <t>risco_condicoes</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Gravidade potencial percebida</t>
+          <t>Condições que podem ampliar dificuldades de proteção (não são características das pessoas — são condições do ambiente/organização)</t>
         </is>
       </c>
       <c r="D44" t="inlineStr"/>
@@ -1603,22 +1599,22 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>risco_grav_just</t>
+          <t>risco_condicoes_outro</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Justificativa da gravidade percebida</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D45" t="inlineStr"/>
       <c r="E45" t="inlineStr"/>
-      <c r="F45" t="inlineStr"/>
-      <c r="G45" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>selected(${risco_condicoes}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr"/>
       <c r="H45" t="inlineStr"/>
       <c r="I45" t="inlineStr"/>
       <c r="J45" t="inlineStr"/>
@@ -1626,27 +1622,23 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>select_one prio_1a5</t>
+          <t>select_multiple cap_resp</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>risco_prioridade</t>
+          <t>risco_capacidades</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Prioridade que a comunidade dá a este risco (1 a 5)</t>
+          <t>Capacidades de resposta já existentes</t>
         </is>
       </c>
       <c r="D46" t="inlineStr"/>
       <c r="E46" t="inlineStr"/>
       <c r="F46" t="inlineStr"/>
-      <c r="G46" t="inlineStr">
-        <is>
-          <t>horizontal-compact</t>
-        </is>
-      </c>
+      <c r="G46" t="inlineStr"/>
       <c r="H46" t="inlineStr"/>
       <c r="I46" t="inlineStr"/>
       <c r="J46" t="inlineStr"/>
@@ -1659,22 +1651,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>risco_evid</t>
+          <t>risco_capacidades_outro</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Evidências associadas</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D47" t="inlineStr"/>
       <c r="E47" t="inlineStr"/>
-      <c r="F47" t="inlineStr"/>
-      <c r="G47" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F47" t="inlineStr">
+        <is>
+          <t>selected(${risco_capacidades}, 'outro')</t>
+        </is>
+      </c>
+      <c r="G47" t="inlineStr"/>
       <c r="H47" t="inlineStr"/>
       <c r="I47" t="inlineStr"/>
       <c r="J47" t="inlineStr"/>
@@ -1682,17 +1674,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>select_multiple marc_risco</t>
+          <t>select_one aval_cap</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>risco_marcacoes</t>
+          <t>risco_aval_cap</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Marcações</t>
+          <t>Avaliação geral da capacidade de resposta</t>
         </is>
       </c>
       <c r="D48" t="inlineStr"/>
@@ -1706,11 +1698,19 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>end_repeat</t>
-        </is>
-      </c>
-      <c r="B49" t="inlineStr"/>
-      <c r="C49" t="inlineStr"/>
+          <t>select_one bma_ns</t>
+        </is>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>risco_prob</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>Probabilidade percebida (não é medição técnica)</t>
+        </is>
+      </c>
       <c r="D49" t="inlineStr"/>
       <c r="E49" t="inlineStr"/>
       <c r="F49" t="inlineStr"/>
@@ -1722,17 +1722,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_one bma_ns</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>cartografia</t>
+          <t>risco_grav</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Cartografia participativa (MAP_*)</t>
+          <t>Gravidade potencial percebida</t>
         </is>
       </c>
       <c r="D50" t="inlineStr"/>
@@ -1746,23 +1746,27 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>map_nota</t>
+          <t>risco_grav_just</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>A cartografia pode registrar zonas de risco, de insegurança, de afeto, recursos/pontos de apoio, lugares de memória e áreas de cuidado/preservação. Esta costuma ser uma etapa que se beneficia de apoio de tutoria — se tiver dúvidas sobre como conduzir a cartografia com a turma/comunidade, procure a equipe de tutoria antes de preencher.</t>
+          <t>Justificativa da gravidade percebida</t>
         </is>
       </c>
       <c r="D51" t="inlineStr"/>
       <c r="E51" t="inlineStr"/>
       <c r="F51" t="inlineStr"/>
-      <c r="G51" t="inlineStr"/>
+      <c r="G51" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H51" t="inlineStr"/>
       <c r="I51" t="inlineStr"/>
       <c r="J51" t="inlineStr"/>
@@ -1770,23 +1774,27 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>select_multiple cartog_quem</t>
+          <t>select_one prio_1a5</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>map_quem</t>
+          <t>risco_prioridade</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Quem participou da cartografia?</t>
+          <t>Prioridade que a comunidade dá a este risco (1 a 5)</t>
         </is>
       </c>
       <c r="D52" t="inlineStr"/>
       <c r="E52" t="inlineStr"/>
       <c r="F52" t="inlineStr"/>
-      <c r="G52" t="inlineStr"/>
+      <c r="G52" t="inlineStr">
+        <is>
+          <t>horizontal-compact</t>
+        </is>
+      </c>
       <c r="H52" t="inlineStr"/>
       <c r="I52" t="inlineStr"/>
       <c r="J52" t="inlineStr"/>
@@ -1799,22 +1807,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>map_quem_outro</t>
+          <t>risco_evid</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Evidências associadas</t>
         </is>
       </c>
       <c r="D53" t="inlineStr"/>
       <c r="E53" t="inlineStr"/>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>selected(${map_quem}, 'outro')</t>
-        </is>
-      </c>
-      <c r="G53" t="inlineStr"/>
+      <c r="F53" t="inlineStr"/>
+      <c r="G53" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H53" t="inlineStr"/>
       <c r="I53" t="inlineStr"/>
       <c r="J53" t="inlineStr"/>
@@ -1822,27 +1830,23 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>select_multiple marc_risco</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>map_novo</t>
+          <t>risco_marcacoes</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>O que a cartografia revelou de novo?</t>
+          <t>Marcações</t>
         </is>
       </c>
       <c r="D54" t="inlineStr"/>
       <c r="E54" t="inlineStr"/>
       <c r="F54" t="inlineStr"/>
-      <c r="G54" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr"/>
       <c r="I54" t="inlineStr"/>
       <c r="J54" t="inlineStr"/>
@@ -1850,19 +1854,11 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>select_one sim_nao_nsabe</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>map_dif</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>Houve diferenças de percepção entre participantes?</t>
-        </is>
-      </c>
+          <t>end_repeat</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr"/>
+      <c r="C55" t="inlineStr"/>
       <c r="D55" t="inlineStr"/>
       <c r="E55" t="inlineStr"/>
       <c r="F55" t="inlineStr"/>
@@ -1874,31 +1870,23 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>map_dif_desc</t>
+          <t>cartografia</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Descreva essas diferenças</t>
+          <t>Cartografia participativa (MAP_*)</t>
         </is>
       </c>
       <c r="D56" t="inlineStr"/>
       <c r="E56" t="inlineStr"/>
-      <c r="F56" t="inlineStr">
-        <is>
-          <t>${map_dif}='sim'</t>
-        </is>
-      </c>
-      <c r="G56" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="F56" t="inlineStr"/>
+      <c r="G56" t="inlineStr"/>
       <c r="H56" t="inlineStr"/>
       <c r="I56" t="inlineStr"/>
       <c r="J56" t="inlineStr"/>
@@ -1906,27 +1894,23 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>map_porque</t>
+          <t>map_nota</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Se a cartografia ainda não foi feita, por quê?</t>
+          <t>A cartografia pode registrar zonas de risco, de insegurança, de afeto, recursos/pontos de apoio, lugares de memória e áreas de cuidado/preservação. Esta costuma ser uma etapa que se beneficia de apoio de tutoria — se tiver dúvidas sobre como conduzir a cartografia com a turma/comunidade, procure a equipe de tutoria antes de preencher.</t>
         </is>
       </c>
       <c r="D57" t="inlineStr"/>
       <c r="E57" t="inlineStr"/>
       <c r="F57" t="inlineStr"/>
-      <c r="G57" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G57" t="inlineStr"/>
       <c r="H57" t="inlineStr"/>
       <c r="I57" t="inlineStr"/>
       <c r="J57" t="inlineStr"/>
@@ -1934,17 +1918,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>image</t>
+          <t>select_multiple cartog_quem</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>map_file</t>
+          <t>map_quem</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Anexar imagem da cartografia (MAP_FILE)</t>
+          <t>Quem participou da cartografia?</t>
         </is>
       </c>
       <c r="D58" t="inlineStr"/>
@@ -1958,14 +1942,26 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr"/>
-      <c r="C59" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>map_quem_outro</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>Especifique (Outro)</t>
+        </is>
+      </c>
       <c r="D59" t="inlineStr"/>
       <c r="E59" t="inlineStr"/>
-      <c r="F59" t="inlineStr"/>
+      <c r="F59" t="inlineStr">
+        <is>
+          <t>selected(${map_quem}, 'outro')</t>
+        </is>
+      </c>
       <c r="G59" t="inlineStr"/>
       <c r="H59" t="inlineStr"/>
       <c r="I59" t="inlineStr"/>
@@ -1974,23 +1970,27 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>begin_repeat</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>evid_e4</t>
+          <t>map_novo</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Evidências — Evidências sobre riscos</t>
+          <t>O que a cartografia revelou de novo?</t>
         </is>
       </c>
       <c r="D60" t="inlineStr"/>
       <c r="E60" t="inlineStr"/>
       <c r="F60" t="inlineStr"/>
-      <c r="G60" t="inlineStr"/>
+      <c r="G60" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H60" t="inlineStr"/>
       <c r="I60" t="inlineStr"/>
       <c r="J60" t="inlineStr"/>
@@ -1998,17 +1998,17 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one sim_nao_nsabe</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>evid_e4_nota</t>
+          <t>map_dif</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
+          <t>Houve diferenças de percepção entre participantes?</t>
         </is>
       </c>
       <c r="D61" t="inlineStr"/>
@@ -2022,23 +2022,31 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>select_one tipo_evid</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>evid_e4_tipo</t>
+          <t>map_dif_desc</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Tipo de evidência</t>
+          <t>Descreva essas diferenças</t>
         </is>
       </c>
       <c r="D62" t="inlineStr"/>
       <c r="E62" t="inlineStr"/>
-      <c r="F62" t="inlineStr"/>
-      <c r="G62" t="inlineStr"/>
+      <c r="F62" t="inlineStr">
+        <is>
+          <t>${map_dif}='sim'</t>
+        </is>
+      </c>
+      <c r="G62" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H62" t="inlineStr"/>
       <c r="I62" t="inlineStr"/>
       <c r="J62" t="inlineStr"/>
@@ -2051,22 +2059,22 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>evid_e4_tipo_outro</t>
+          <t>map_porque</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Especifique (Outro)</t>
+          <t>Se a cartografia ainda não foi feita, por quê?</t>
         </is>
       </c>
       <c r="D63" t="inlineStr"/>
       <c r="E63" t="inlineStr"/>
-      <c r="F63" t="inlineStr">
-        <is>
-          <t>${evid_e4_tipo}='outro'</t>
-        </is>
-      </c>
-      <c r="G63" t="inlineStr"/>
+      <c r="F63" t="inlineStr"/>
+      <c r="G63" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H63" t="inlineStr"/>
       <c r="I63" t="inlineStr"/>
       <c r="J63" t="inlineStr"/>
@@ -2074,27 +2082,23 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>image</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>evid_e4_desc</t>
+          <t>map_file</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Descreva a evidência</t>
+          <t>Anexar imagem da cartografia (MAP_FILE)</t>
         </is>
       </c>
       <c r="D64" t="inlineStr"/>
       <c r="E64" t="inlineStr"/>
       <c r="F64" t="inlineStr"/>
-      <c r="G64" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G64" t="inlineStr"/>
       <c r="H64" t="inlineStr"/>
       <c r="I64" t="inlineStr"/>
       <c r="J64" t="inlineStr"/>
@@ -2102,19 +2106,11 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>file</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>evid_e4_anexo</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>Anexo (foto/documento) — opcional</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr"/>
+      <c r="C65" t="inlineStr"/>
       <c r="D65" t="inlineStr"/>
       <c r="E65" t="inlineStr"/>
       <c r="F65" t="inlineStr"/>
@@ -2126,11 +2122,19 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>end_repeat</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr"/>
-      <c r="C66" t="inlineStr"/>
+          <t>begin_repeat</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>evid_e4</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Evidências — Evidências sobre riscos</t>
+        </is>
+      </c>
       <c r="D66" t="inlineStr"/>
       <c r="E66" t="inlineStr"/>
       <c r="F66" t="inlineStr"/>
@@ -2142,11 +2146,19 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr"/>
-      <c r="C67" t="inlineStr"/>
+          <t>note</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>evid_e4_nota</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Evidências sustentam análises futuras (problemas, prioridades, plano de ação). Registrar não é obrigatório para todo campo, mas fortalece a rastreabilidade do diagnóstico.</t>
+        </is>
+      </c>
       <c r="D67" t="inlineStr"/>
       <c r="E67" t="inlineStr"/>
       <c r="F67" t="inlineStr"/>
@@ -2158,17 +2170,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>begin_group</t>
+          <t>select_one tipo_evid</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>etapa5</t>
+          <t>evid_e4_tipo</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Etapa 5 — Leitura Integrada (FOFA)</t>
+          <t>Tipo de evidência</t>
         </is>
       </c>
       <c r="D68" t="inlineStr"/>
@@ -2182,22 +2194,26 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>e5_nota</t>
+          <t>evid_e4_tipo_outro</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>No sistema original esta matriz é alimentada automaticamente pelas etapas anteriores (principalmente Riscos e Participação e Redes). No Kobo, preencha manualmente a partir das respostas já registradas (tutoria pode ajudar). Nada é definitivo sem revisão humana.</t>
+          <t>Especifique (Outro)</t>
         </is>
       </c>
       <c r="D69" t="inlineStr"/>
       <c r="E69" t="inlineStr"/>
-      <c r="F69" t="inlineStr"/>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>${evid_e4_tipo}='outro'</t>
+        </is>
+      </c>
       <c r="G69" t="inlineStr"/>
       <c r="H69" t="inlineStr"/>
       <c r="I69" t="inlineStr"/>
@@ -2206,27 +2222,27 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>select_one sim_nao_ns</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>q5_1</t>
+          <t>evid_e4_desc</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Q5.1. A leitura construída até aqui reflete bem a realidade do local e do território?</t>
+          <t>Descreva a evidência</t>
         </is>
       </c>
       <c r="D70" t="inlineStr"/>
-      <c r="E70" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
-      </c>
+      <c r="E70" t="inlineStr"/>
       <c r="F70" t="inlineStr"/>
-      <c r="G70" t="inlineStr"/>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H70" t="inlineStr"/>
       <c r="I70" t="inlineStr"/>
       <c r="J70" t="inlineStr"/>
@@ -2234,27 +2250,23 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>file</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>q5_2</t>
+          <t>evid_e4_anexo</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Q5.2. Algum contexto importante para interpretar esta leitura integrada?</t>
+          <t>Anexo (foto/documento) — opcional</t>
         </is>
       </c>
       <c r="D71" t="inlineStr"/>
       <c r="E71" t="inlineStr"/>
       <c r="F71" t="inlineStr"/>
-      <c r="G71" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G71" t="inlineStr"/>
       <c r="H71" t="inlineStr"/>
       <c r="I71" t="inlineStr"/>
       <c r="J71" t="inlineStr"/>
@@ -2262,27 +2274,15 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B72" t="inlineStr">
-        <is>
-          <t>swot_forcas</t>
-        </is>
-      </c>
-      <c r="C72" t="inlineStr">
-        <is>
-          <t>Forças — adicione uma por linha</t>
-        </is>
-      </c>
+          <t>end_repeat</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr"/>
+      <c r="C72" t="inlineStr"/>
       <c r="D72" t="inlineStr"/>
       <c r="E72" t="inlineStr"/>
       <c r="F72" t="inlineStr"/>
-      <c r="G72" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G72" t="inlineStr"/>
       <c r="H72" t="inlineStr"/>
       <c r="I72" t="inlineStr"/>
       <c r="J72" t="inlineStr"/>
@@ -2290,27 +2290,15 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B73" t="inlineStr">
-        <is>
-          <t>swot_fragilidades</t>
-        </is>
-      </c>
-      <c r="C73" t="inlineStr">
-        <is>
-          <t>Fragilidades — adicione uma por linha</t>
-        </is>
-      </c>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr"/>
+      <c r="C73" t="inlineStr"/>
       <c r="D73" t="inlineStr"/>
       <c r="E73" t="inlineStr"/>
       <c r="F73" t="inlineStr"/>
-      <c r="G73" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G73" t="inlineStr"/>
       <c r="H73" t="inlineStr"/>
       <c r="I73" t="inlineStr"/>
       <c r="J73" t="inlineStr"/>
@@ -2318,27 +2306,23 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>begin_group</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>swot_oportunidades</t>
+          <t>etapa5</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Oportunidades — adicione uma por linha</t>
+          <t>Etapa 5 — Leitura Integrada (FOFA)</t>
         </is>
       </c>
       <c r="D74" t="inlineStr"/>
       <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
-      <c r="G74" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G74" t="inlineStr"/>
       <c r="H74" t="inlineStr"/>
       <c r="I74" t="inlineStr"/>
       <c r="J74" t="inlineStr"/>
@@ -2346,27 +2330,23 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>swot_ameacas</t>
+          <t>e5_nota</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Ameaças — adicione uma por linha</t>
+          <t>No sistema original esta matriz é alimentada automaticamente pelas etapas anteriores (principalmente Riscos e Participação e Redes). No Kobo, preencha manualmente a partir das respostas já registradas (tutoria pode ajudar). Nada é definitivo sem revisão humana.</t>
         </is>
       </c>
       <c r="D75" t="inlineStr"/>
       <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
-      <c r="G75" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G75" t="inlineStr"/>
       <c r="H75" t="inlineStr"/>
       <c r="I75" t="inlineStr"/>
       <c r="J75" t="inlineStr"/>
@@ -2374,21 +2354,25 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>select_one sim_nao_ns</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>swot_rel_nota</t>
+          <t>q5_1</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Relações estratégicas</t>
+          <t>Q5.1. A leitura construída até aqui reflete bem a realidade do local e do território?</t>
         </is>
       </c>
       <c r="D76" t="inlineStr"/>
-      <c r="E76" t="inlineStr"/>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
       <c r="H76" t="inlineStr"/>
@@ -2403,12 +2387,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>swot_rel_forca_ameaca</t>
+          <t>q5_2</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Como uma força pode responder a uma ameaça? (SWOT_REL_STRENGTH_THREAT)</t>
+          <t>Q5.2. Algum contexto importante para interpretar esta leitura integrada?</t>
         </is>
       </c>
       <c r="D77" t="inlineStr"/>
@@ -2431,12 +2415,12 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>swot_rel_oport_fragil</t>
+          <t>swot_forcas</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Como uma oportunidade pode reduzir uma fragilidade? (SWOT_REL_OPPORTUNITY_WEAKNESS)</t>
+          <t>Forças — adicione uma por linha</t>
         </is>
       </c>
       <c r="D78" t="inlineStr"/>
@@ -2459,12 +2443,12 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>swot_rel_fragil_ameaca</t>
+          <t>swot_fragilidades</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Como uma fragilidade agrava uma ameaça? (SWOT_REL_WEAKNESS_THREAT)</t>
+          <t>Fragilidades — adicione uma por linha</t>
         </is>
       </c>
       <c r="D79" t="inlineStr"/>
@@ -2482,23 +2466,27 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>note</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>cap_nota</t>
+          <t>swot_oportunidades</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Capacidades adaptativas: são recursos, saberes e formas de organização que o local e o território JÁ possuem e que ajudam a responder a desafios socioambientais e climáticos. Capacidades comunitárias não são tratadas como inferiores às institucionais — registre o que já existe, mesmo que informal.</t>
+          <t>Oportunidades — adicione uma por linha</t>
         </is>
       </c>
       <c r="D80" t="inlineStr"/>
       <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
-      <c r="G80" t="inlineStr"/>
+      <c r="G80" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H80" t="inlineStr"/>
       <c r="I80" t="inlineStr"/>
       <c r="J80" t="inlineStr"/>
@@ -2511,19 +2499,15 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>cap_pedagogical</t>
+          <t>swot_ameacas</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Pedagógicas (CAP_PEDAGOGICAL)</t>
-        </is>
-      </c>
-      <c r="D81" t="inlineStr">
-        <is>
-          <t>Saberes e práticas de ensino já disponíveis neste local — ex.: professores com experiência em projetos interdisciplinares, metodologias ativas, uso do território como espaço de aprendizagem.</t>
-        </is>
-      </c>
+          <t>Ameaças — adicione uma por linha</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr"/>
       <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
@@ -2538,31 +2522,23 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>cap_social</t>
+          <t>swot_rel_nota</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Sociais (CAP_SOCIAL)</t>
-        </is>
-      </c>
-      <c r="D82" t="inlineStr">
-        <is>
-          <t>Formas de organização e mobilização das pessoas — ex.: participação estudantil ativa, rede de apoio entre famílias, mutirões, associações comunitárias.</t>
-        </is>
-      </c>
+          <t>Relações estratégicas</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr"/>
       <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
-      <c r="G82" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G82" t="inlineStr"/>
       <c r="H82" t="inlineStr"/>
       <c r="I82" t="inlineStr"/>
       <c r="J82" t="inlineStr"/>
@@ -2575,19 +2551,15 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>cap_institutional</t>
+          <t>swot_rel_forca_ameaca</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Institucionais (CAP_INSTITUTIONAL)</t>
-        </is>
-      </c>
-      <c r="D83" t="inlineStr">
-        <is>
-          <t>Estruturas, normas e gestão do próprio local — ex.: apoio da direção, PPP que sustenta continuidade, canais de decisão coletiva.</t>
-        </is>
-      </c>
+          <t>Como uma força pode responder a uma ameaça? (SWOT_REL_STRENGTH_THREAT)</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr"/>
       <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
       <c r="G83" t="inlineStr">
@@ -2607,19 +2579,15 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>cap_territorial</t>
+          <t>swot_rel_oport_fragil</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Territoriais (CAP_TERRITORIAL)</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>Recursos e conhecimentos do entorno — ex.: conhecimento tradicional sobre o clima local, parceiros no bairro, espaços públicos de apoio.</t>
-        </is>
-      </c>
+          <t>Como uma oportunidade pode reduzir uma fragilidade? (SWOT_REL_OPPORTUNITY_WEAKNESS)</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr"/>
       <c r="E84" t="inlineStr"/>
       <c r="F84" t="inlineStr"/>
       <c r="G84" t="inlineStr">
@@ -2639,19 +2607,15 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>cap_material</t>
+          <t>swot_rel_fragil_ameaca</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Materiais (CAP_MATERIAL)</t>
-        </is>
-      </c>
-      <c r="D85" t="inlineStr">
-        <is>
-          <t>Infraestrutura, equipamentos e recursos físicos — ex.: espaço para horta, materiais didáticos próprios, equipamentos disponíveis.</t>
-        </is>
-      </c>
+          <t>Como uma fragilidade agrava uma ameaça? (SWOT_REL_WEAKNESS_THREAT)</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr"/>
       <c r="E85" t="inlineStr"/>
       <c r="F85" t="inlineStr"/>
       <c r="G85" t="inlineStr">
@@ -2666,27 +2630,23 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>text</t>
+          <t>note</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>q5_3</t>
+          <t>cap_nota</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Q5.3. Qual a principal capacidade do local/comunidade hoje?</t>
+          <t>Capacidades adaptativas: são recursos, saberes e formas de organização que o local e o território JÁ possuem e que ajudam a responder a desafios socioambientais e climáticos. Capacidades comunitárias não são tratadas como inferiores às institucionais — registre o que já existe, mesmo que informal.</t>
         </is>
       </c>
       <c r="D86" t="inlineStr"/>
       <c r="E86" t="inlineStr"/>
       <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr">
-        <is>
-          <t>multiline</t>
-        </is>
-      </c>
+      <c r="G86" t="inlineStr"/>
       <c r="H86" t="inlineStr"/>
       <c r="I86" t="inlineStr"/>
       <c r="J86" t="inlineStr"/>
@@ -2699,15 +2659,19 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>q5_4</t>
+          <t>cap_pedagogical</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Q5.4. Qual a principal limitação hoje?</t>
-        </is>
-      </c>
-      <c r="D87" t="inlineStr"/>
+          <t>Pedagógicas (CAP_PEDAGOGICAL)</t>
+        </is>
+      </c>
+      <c r="D87" t="inlineStr">
+        <is>
+          <t>Saberes e práticas de ensino já disponíveis neste local — ex.: professores com experiência em projetos interdisciplinares, metodologias ativas, uso do território como espaço de aprendizagem.</t>
+        </is>
+      </c>
       <c r="E87" t="inlineStr"/>
       <c r="F87" t="inlineStr"/>
       <c r="G87" t="inlineStr">
@@ -2727,15 +2691,19 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>q5_5</t>
+          <t>cap_social</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Q5.5. Existe alguma oportunidade pouco aproveitada até agora?</t>
-        </is>
-      </c>
-      <c r="D88" t="inlineStr"/>
+          <t>Sociais (CAP_SOCIAL)</t>
+        </is>
+      </c>
+      <c r="D88" t="inlineStr">
+        <is>
+          <t>Formas de organização e mobilização das pessoas — ex.: participação estudantil ativa, rede de apoio entre famílias, mutirões, associações comunitárias.</t>
+        </is>
+      </c>
       <c r="E88" t="inlineStr"/>
       <c r="F88" t="inlineStr"/>
       <c r="G88" t="inlineStr">
@@ -2750,18 +2718,214 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>end_group</t>
-        </is>
-      </c>
-      <c r="B89" t="inlineStr"/>
-      <c r="C89" t="inlineStr"/>
-      <c r="D89" t="inlineStr"/>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>cap_institutional</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>Institucionais (CAP_INSTITUTIONAL)</t>
+        </is>
+      </c>
+      <c r="D89" t="inlineStr">
+        <is>
+          <t>Estruturas, normas e gestão do próprio local — ex.: apoio da direção, PPP que sustenta continuidade, canais de decisão coletiva.</t>
+        </is>
+      </c>
       <c r="E89" t="inlineStr"/>
       <c r="F89" t="inlineStr"/>
-      <c r="G89" t="inlineStr"/>
+      <c r="G89" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
       <c r="H89" t="inlineStr"/>
       <c r="I89" t="inlineStr"/>
       <c r="J89" t="inlineStr"/>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>cap_territorial</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>Territoriais (CAP_TERRITORIAL)</t>
+        </is>
+      </c>
+      <c r="D90" t="inlineStr">
+        <is>
+          <t>Recursos e conhecimentos do entorno — ex.: conhecimento tradicional sobre o clima local, parceiros no bairro, espaços públicos de apoio.</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr"/>
+      <c r="J90" t="inlineStr"/>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>cap_material</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>Materiais (CAP_MATERIAL)</t>
+        </is>
+      </c>
+      <c r="D91" t="inlineStr">
+        <is>
+          <t>Infraestrutura, equipamentos e recursos físicos — ex.: espaço para horta, materiais didáticos próprios, equipamentos disponíveis.</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr"/>
+      <c r="J91" t="inlineStr"/>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>q5_3</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>Q5.3. Qual a principal capacidade do local/comunidade hoje?</t>
+        </is>
+      </c>
+      <c r="D92" t="inlineStr"/>
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr"/>
+      <c r="J92" t="inlineStr"/>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>q5_4</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>Q5.4. Qual a principal limitação hoje?</t>
+        </is>
+      </c>
+      <c r="D93" t="inlineStr"/>
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr"/>
+      <c r="J93" t="inlineStr"/>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>text</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>q5_5</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>Q5.5. Existe alguma oportunidade pouco aproveitada até agora?</t>
+        </is>
+      </c>
+      <c r="D94" t="inlineStr"/>
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
+        <is>
+          <t>multiline</t>
+        </is>
+      </c>
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr"/>
+      <c r="J94" t="inlineStr"/>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr"/>
+      <c r="C95" t="inlineStr"/>
+      <c r="D95" t="inlineStr"/>
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr"/>
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr"/>
+      <c r="J95" t="inlineStr"/>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>end_group</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr"/>
+      <c r="C96" t="inlineStr"/>
+      <c r="D96" t="inlineStr"/>
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr"/>
+      <c r="J96" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2774,7 +2938,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C112"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2797,34 +2961,34 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>sim_nao_ns</t>
+          <t>concordo</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>concordo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Sim, concordo em participar</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>sim_nao_ns</t>
+          <t>concordo</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>nao_concordo</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Não concordo</t>
         </is>
       </c>
     </row>
@@ -2836,46 +3000,46 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>nao_sabemos</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Não sabemos</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>sim_nao_nsabe</t>
+          <t>sim_nao_ns</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>sim</t>
+          <t>nao</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Sim</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>sim_nao_nsabe</t>
+          <t>sim_nao_ns</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>nao</t>
+          <t>nao_sabemos</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Não</t>
+          <t>Não sabemos</t>
         </is>
       </c>
     </row>
@@ -2887,46 +3051,46 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>sim</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Sim</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>tipo_evid</t>
+          <t>sim_nao_nsabe</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>observacao_direta</t>
+          <t>nao</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Observação direta</t>
+          <t>Não</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>tipo_evid</t>
+          <t>sim_nao_nsabe</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>documento</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Documento</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -2938,12 +3102,12 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>foto</t>
+          <t>observacao_direta</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Foto</t>
+          <t>Observação direta</t>
         </is>
       </c>
     </row>
@@ -2955,12 +3119,12 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>depoimento</t>
+          <t>documento</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Depoimento</t>
+          <t>Documento</t>
         </is>
       </c>
     </row>
@@ -2972,12 +3136,12 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>registro_historico</t>
+          <t>foto</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Registro histórico</t>
+          <t>Foto</t>
         </is>
       </c>
     </row>
@@ -2989,46 +3153,46 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>depoimento</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Depoimento</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>ameacas</t>
+          <t>tipo_evid</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>enchente</t>
+          <t>registro_historico</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Enchente</t>
+          <t>Registro histórico</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>ameacas</t>
+          <t>tipo_evid</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>inundacao</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Inundação</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
@@ -3040,12 +3204,12 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>alagamento</t>
+          <t>enchente</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Alagamento</t>
+          <t>Enchente</t>
         </is>
       </c>
     </row>
@@ -3057,12 +3221,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>enxurrada</t>
+          <t>inundacao</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Enxurrada</t>
+          <t>Inundação</t>
         </is>
       </c>
     </row>
@@ -3074,12 +3238,12 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>deslizamento</t>
+          <t>alagamento</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Deslizamento</t>
+          <t>Alagamento</t>
         </is>
       </c>
     </row>
@@ -3091,12 +3255,12 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>erosao</t>
+          <t>enxurrada</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Erosão</t>
+          <t>Enxurrada</t>
         </is>
       </c>
     </row>
@@ -3108,12 +3272,12 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>estiagem_seca</t>
+          <t>deslizamento</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>Estiagem/seca</t>
+          <t>Deslizamento</t>
         </is>
       </c>
     </row>
@@ -3125,12 +3289,12 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>falta_de_agua</t>
+          <t>erosao</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Falta de água</t>
+          <t>Erosão</t>
         </is>
       </c>
     </row>
@@ -3142,12 +3306,12 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>onda_de_calor</t>
+          <t>estiagem_seca</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Onda de calor</t>
+          <t>Estiagem/seca</t>
         </is>
       </c>
     </row>
@@ -3159,12 +3323,12 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>frio_intenso</t>
+          <t>falta_de_agua</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Frio intenso</t>
+          <t>Falta de água</t>
         </is>
       </c>
     </row>
@@ -3176,12 +3340,12 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>tempestades</t>
+          <t>onda_de_calor</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Tempestades</t>
+          <t>Onda de calor</t>
         </is>
       </c>
     </row>
@@ -3193,12 +3357,12 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>vendavais</t>
+          <t>frio_intenso</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Vendavais</t>
+          <t>Frio intenso</t>
         </is>
       </c>
     </row>
@@ -3210,12 +3374,12 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>granizo</t>
+          <t>tempestades</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Granizo</t>
+          <t>Tempestades</t>
         </is>
       </c>
     </row>
@@ -3227,12 +3391,12 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>ciclones</t>
+          <t>vendavais</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ciclones</t>
+          <t>Vendavais</t>
         </is>
       </c>
     </row>
@@ -3244,12 +3408,12 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>queimadas</t>
+          <t>granizo</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Queimadas</t>
+          <t>Granizo</t>
         </is>
       </c>
     </row>
@@ -3261,12 +3425,12 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>incendios</t>
+          <t>ciclones</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Incêndios</t>
+          <t>Ciclones</t>
         </is>
       </c>
     </row>
@@ -3278,12 +3442,12 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>fumaca_poluicao_atmosferica</t>
+          <t>queimadas</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Fumaça/poluição atmosférica</t>
+          <t>Queimadas</t>
         </is>
       </c>
     </row>
@@ -3295,12 +3459,12 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>contaminacao_da_agua</t>
+          <t>incendios</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Contaminação da água</t>
+          <t>Incêndios</t>
         </is>
       </c>
     </row>
@@ -3312,12 +3476,12 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>problemas_relacionados_a_residuo</t>
+          <t>fumaca_poluicao_atmosferica</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Problemas relacionados a resíduos</t>
+          <t>Fumaça/poluição atmosférica</t>
         </is>
       </c>
     </row>
@@ -3329,46 +3493,46 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>contaminacao_da_agua</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Outros</t>
+          <t>Contaminação da água</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>base_percepcao</t>
+          <t>ameacas</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>observacao_ao_longo_dos_anos</t>
+          <t>problemas_relacionados_a_residuo</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Observação ao longo dos anos</t>
+          <t>Problemas relacionados a resíduos</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>base_percepcao</t>
+          <t>ameacas</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>relatos_de_moradores_antigos</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Relatos de moradores antigos</t>
+          <t>Outros</t>
         </is>
       </c>
     </row>
@@ -3380,12 +3544,12 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>comparacao_com_registros</t>
+          <t>observacao_ao_longo_dos_anos</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Comparação com registros</t>
+          <t>Observação ao longo dos anos</t>
         </is>
       </c>
     </row>
@@ -3397,12 +3561,12 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>noticias</t>
+          <t>relatos_de_moradores_antigos</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Notícias</t>
+          <t>Relatos de moradores antigos</t>
         </is>
       </c>
     </row>
@@ -3414,46 +3578,46 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>comparacao_com_registros</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Comparação com registros</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>fontes_risco</t>
+          <t>base_percepcao</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>defesa_civil</t>
+          <t>noticias</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Defesa Civil</t>
+          <t>Notícias</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>fontes_risco</t>
+          <t>base_percepcao</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>dados_meteorologicos</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Dados meteorológicos (ex.: INMET)</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -3465,12 +3629,12 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>universidade</t>
+          <t>defesa_civil</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Universidade</t>
+          <t>Defesa Civil</t>
         </is>
       </c>
     </row>
@@ -3482,12 +3646,12 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ong</t>
+          <t>dados_meteorologicos</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ONG</t>
+          <t>Dados meteorológicos (ex.: INMET)</t>
         </is>
       </c>
     </row>
@@ -3499,12 +3663,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>conhecimento_tradicional</t>
+          <t>universidade</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Conhecimento tradicional</t>
+          <t>Universidade</t>
         </is>
       </c>
     </row>
@@ -3516,12 +3680,12 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>nao_ha_fonte_consultada</t>
+          <t>ong</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Não há fonte consultada</t>
+          <t>ONG</t>
         </is>
       </c>
     </row>
@@ -3533,46 +3697,46 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>conhecimento_tradicional</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Conhecimento tradicional</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>afetou</t>
+          <t>fontes_risco</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>escola</t>
+          <t>nao_ha_fonte_consultada</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Local</t>
+          <t>Não há fonte consultada</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>afetou</t>
+          <t>fontes_risco</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>comunidade</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Comunidade</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
@@ -3584,12 +3748,12 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>ambos</t>
+          <t>escola</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ambos</t>
+          <t>Local</t>
         </is>
       </c>
     </row>
@@ -3601,12 +3765,12 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>nenhum</t>
+          <t>comunidade</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Nenhum</t>
+          <t>Comunidade</t>
         </is>
       </c>
     </row>
@@ -3618,46 +3782,46 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>ambos</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Ambos</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>freq_risco</t>
+          <t>afetou</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>raro</t>
+          <t>nenhum</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Raro (já ocorreu uma vez)</t>
+          <t>Nenhum</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>freq_risco</t>
+          <t>afetou</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ocasional</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Ocasional</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -3669,12 +3833,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>frequente</t>
+          <t>raro</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Frequente</t>
+          <t>Raro (já ocorreu uma vez)</t>
         </is>
       </c>
     </row>
@@ -3686,12 +3850,12 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>muito_frequente_recorrente</t>
+          <t>ocasional</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Muito frequente/recorrente</t>
+          <t>Ocasional</t>
         </is>
       </c>
     </row>
@@ -3703,46 +3867,46 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>frequente</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Frequente</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>impacto_risco</t>
+          <t>freq_risco</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>interrupcao_de_aulas</t>
+          <t>muito_frequente_recorrente</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Interrupção de aulas</t>
+          <t>Muito frequente/recorrente</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>impacto_risco</t>
+          <t>freq_risco</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>danos_a_estrutura</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Danos à estrutura</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -3754,12 +3918,12 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>acesso_interrompido</t>
+          <t>interrupcao_de_aulas</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Acesso interrompido</t>
+          <t>Interrupção de aulas</t>
         </is>
       </c>
     </row>
@@ -3771,12 +3935,12 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>perda_de_materiais</t>
+          <t>danos_a_estrutura</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Perda de materiais</t>
+          <t>Danos à estrutura</t>
         </is>
       </c>
     </row>
@@ -3788,12 +3952,12 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>impacto_na_saude</t>
+          <t>acesso_interrompido</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Impacto na saúde</t>
+          <t>Acesso interrompido</t>
         </is>
       </c>
     </row>
@@ -3805,12 +3969,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>impacto_emocional</t>
+          <t>perda_de_materiais</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Impacto emocional</t>
+          <t>Perda de materiais</t>
         </is>
       </c>
     </row>
@@ -3822,46 +3986,46 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>impacto_na_saude</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Impacto na saúde</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>ativos</t>
+          <t>impacto_risco</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>predio_escolar</t>
+          <t>impacto_emocional</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Prédio escolar</t>
+          <t>Impacto emocional</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>ativos</t>
+          <t>impacto_risco</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>biblioteca</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>Biblioteca</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -3873,12 +4037,12 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>quadra</t>
+          <t>predio_escolar</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Quadra</t>
+          <t>Prédio escolar</t>
         </is>
       </c>
     </row>
@@ -3890,12 +4054,12 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>horta</t>
+          <t>biblioteca</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Horta</t>
+          <t>Biblioteca</t>
         </is>
       </c>
     </row>
@@ -3907,12 +4071,12 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>equipamentos</t>
+          <t>quadra</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Equipamentos</t>
+          <t>Quadra</t>
         </is>
       </c>
     </row>
@@ -3924,12 +4088,12 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>arquivos_documentos</t>
+          <t>horta</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Arquivos/documentos</t>
+          <t>Horta</t>
         </is>
       </c>
     </row>
@@ -3941,46 +4105,46 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>equipamentos</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Equipamentos</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>grupos_exp</t>
+          <t>ativos</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>estudantes</t>
+          <t>arquivos_documentos</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Estudantes</t>
+          <t>Arquivos/documentos</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>grupos_exp</t>
+          <t>ativos</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>professores</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Professores(as)</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -3992,12 +4156,12 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>funcionarios</t>
+          <t>estudantes</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Funcionários(as)</t>
+          <t>Estudantes</t>
         </is>
       </c>
     </row>
@@ -4009,12 +4173,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>familias</t>
+          <t>professores</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Famílias</t>
+          <t>Professores(as)</t>
         </is>
       </c>
     </row>
@@ -4026,12 +4190,12 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>pessoas_com_deficiencia</t>
+          <t>funcionarios</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Pessoas com deficiência</t>
+          <t>Funcionários(as)</t>
         </is>
       </c>
     </row>
@@ -4043,12 +4207,12 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>criancas_pequenas</t>
+          <t>familias</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Crianças pequenas</t>
+          <t>Famílias</t>
         </is>
       </c>
     </row>
@@ -4060,12 +4224,12 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>idosos</t>
+          <t>pessoas_com_deficiencia</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Idosos</t>
+          <t>Pessoas com deficiência</t>
         </is>
       </c>
     </row>
@@ -4077,46 +4241,46 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>criancas_pequenas</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Outro</t>
+          <t>Crianças pequenas</t>
         </is>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>cond_amplia</t>
+          <t>grupos_exp</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>acessibilidade_limitada_nas_rota</t>
+          <t>idosos</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>Acessibilidade limitada nas rotas de saída</t>
+          <t>Idosos</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>cond_amplia</t>
+          <t>grupos_exp</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>ausencia_de_sinalizacao_de_emerg</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Ausência de sinalização de emergência</t>
+          <t>Outro</t>
         </is>
       </c>
     </row>
@@ -4128,12 +4292,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>estrutura_fisica_fragilizada</t>
+          <t>acessibilidade_limitada_nas_rota</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Estrutura física fragilizada</t>
+          <t>Acessibilidade limitada nas rotas de saída</t>
         </is>
       </c>
     </row>
@@ -4145,12 +4309,12 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>ausencia_de_comunicacao_acessive</t>
+          <t>ausencia_de_sinalizacao_de_emerg</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Ausência de comunicação acessível (Libras/Braile/linguagem simples)</t>
+          <t>Ausência de sinalização de emergência</t>
         </is>
       </c>
     </row>
@@ -4162,12 +4326,12 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>ausencia_de_plano_de_evacuacao_a</t>
+          <t>estrutura_fisica_fragilizada</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Ausência de plano de evacuação adaptado</t>
+          <t>Estrutura física fragilizada</t>
         </is>
       </c>
     </row>
@@ -4179,12 +4343,12 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>distancia_de_pontos_de_apoio_soc</t>
+          <t>ausencia_de_comunicacao_acessive</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Distância de pontos de apoio/socorro</t>
+          <t>Ausência de comunicação acessível (Libras/Braile/linguagem simples)</t>
         </is>
       </c>
     </row>
@@ -4196,46 +4360,46 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>ausencia_de_plano_de_evacuacao_a</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Outra condição</t>
+          <t>Ausência de plano de evacuação adaptado</t>
         </is>
       </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>cap_resp</t>
+          <t>cond_amplia</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>brigada_equipe_treinada</t>
+          <t>distancia_de_pontos_de_apoio_soc</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Brigada/equipe treinada</t>
+          <t>Distância de pontos de apoio/socorro</t>
         </is>
       </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>cap_resp</t>
+          <t>cond_amplia</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>plano_de_evacuacao</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Plano de evacuação</t>
+          <t>Outra condição</t>
         </is>
       </c>
     </row>
@@ -4247,12 +4411,12 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>comunicacao_de_alerta</t>
+          <t>brigada_equipe_treinada</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Comunicação de alerta</t>
+          <t>Brigada/equipe treinada</t>
         </is>
       </c>
     </row>
@@ -4264,12 +4428,12 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>apoio_de_rede_externa</t>
+          <t>plano_de_evacuacao</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>Apoio de rede externa</t>
+          <t>Plano de evacuação</t>
         </is>
       </c>
     </row>
@@ -4281,12 +4445,12 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>kit_de_emergencia</t>
+          <t>comunicacao_de_alerta</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Kit de emergência</t>
+          <t>Comunicação de alerta</t>
         </is>
       </c>
     </row>
@@ -4298,12 +4462,12 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>nenhuma_identificada</t>
+          <t>apoio_de_rede_externa</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Nenhuma identificada</t>
+          <t>Apoio de rede externa</t>
         </is>
       </c>
     </row>
@@ -4315,46 +4479,46 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>outro</t>
+          <t>kit_de_emergencia</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Outra</t>
+          <t>Kit de emergência</t>
         </is>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>aval_cap</t>
+          <t>cap_resp</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>boa</t>
+          <t>nenhuma_identificada</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Boa</t>
+          <t>Nenhuma identificada</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>aval_cap</t>
+          <t>cap_resp</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>regular</t>
+          <t>outro</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Regular</t>
+          <t>Outra</t>
         </is>
       </c>
     </row>
@@ -4366,12 +4530,12 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>fraca</t>
+          <t>boa</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Fraca</t>
+          <t>Boa</t>
         </is>
       </c>
     </row>
@@ -4383,12 +4547,12 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>inexistente</t>
+          <t>regular</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Inexistente</t>
+          <t>Regular</t>
         </is>
       </c>
     </row>
@@ -4400,46 +4564,46 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>fraca</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Fraca</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>bma_ns</t>
+          <t>aval_cap</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>baixa</t>
+          <t>inexistente</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>Baixa</t>
+          <t>Inexistente</t>
         </is>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>bma_ns</t>
+          <t>aval_cap</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>media</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Média</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -4451,12 +4615,12 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>alta</t>
+          <t>baixa</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Alta</t>
+          <t>Baixa</t>
         </is>
       </c>
     </row>
@@ -4468,46 +4632,46 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>nao_sabe</t>
+          <t>media</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>Não sabe</t>
+          <t>Média</t>
         </is>
       </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>prio_1a5</t>
+          <t>bma_ns</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>alta</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>1 — Muito baixa</t>
+          <t>Alta</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>prio_1a5</t>
+          <t>bma_ns</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>nao_sabe</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>Não sabe</t>
         </is>
       </c>
     </row>
@@ -4519,12 +4683,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>3</t>
+          <t>1</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>3 — Média</t>
+          <t>1 — Muito baixa</t>
         </is>
       </c>
     </row>
@@ -4536,12 +4700,12 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>2</t>
         </is>
       </c>
     </row>
@@ -4553,46 +4717,46 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>3</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>5 — Muito alta</t>
+          <t>3 — Média</t>
         </is>
       </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>marc_risco</t>
+          <t>prio_1a5</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>lacuna</t>
+          <t>4</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Não sabemos avaliar isso com segurança (gera lacuna de conhecimento)</t>
+          <t>4</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>marc_risco</t>
+          <t>prio_1a5</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>aval_externa</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Requer avaliação técnica externa</t>
+          <t>5 — Muito alta</t>
         </is>
       </c>
     </row>
@@ -4604,46 +4768,46 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>selecionado</t>
+          <t>lacuna</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Selecionar este risco para a Leitura Integrada e planejamento</t>
+          <t>Não sabemos avaliar isso com segurança (gera lacuna de conhecimento)</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>cartog_quem</t>
+          <t>marc_risco</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>estudantes</t>
+          <t>aval_externa</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Estudantes</t>
+          <t>Requer avaliação técnica externa</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>cartog_quem</t>
+          <t>marc_risco</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>professores</t>
+          <t>selecionado</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Professores(as)</t>
+          <t>Selecionar este risco para a Leitura Integrada e planejamento</t>
         </is>
       </c>
     </row>
@@ -4655,12 +4819,12 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>comunidade</t>
+          <t>estudantes</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Comunidade</t>
+          <t>Estudantes</t>
         </is>
       </c>
     </row>
@@ -4672,10 +4836,44 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
+          <t>professores</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>Professores(as)</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>cartog_quem</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>comunidade</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>Comunidade</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>cartog_quem</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
           <t>outro</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C114" t="inlineStr">
         <is>
           <t>Outros</t>
         </is>
@@ -4745,7 +4943,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>pages</t>
+          <t>theme-grid no-text-transform</t>
         </is>
       </c>
     </row>

</xml_diff>